<commit_message>
scan: seg7 2026-06-17 19:27 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-06-17.xlsx
+++ b/output/full_scan/batch_seq8_2026-06-17.xlsx
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>219.2215053486098</v>
+        <v>219.2215053486097</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>44.15</v>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>204.2618175993962</v>
+        <v>204.2618175993961</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>61.7</v>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>201.3616751267398</v>
+        <v>201.3616751267397</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>61.2</v>

</xml_diff>